<commit_message>
Fixed data error (lamu mainland)
</commit_message>
<xml_diff>
--- a/AIMMSProject/data/VS_5Vessel_15Cargo.xlsx
+++ b/AIMMSProject/data/VS_5Vessel_15Cargo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\u\s\examples\application-examples\vessel-scheduling\AIMMS Project\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\u\s\examples\application-examples\vessel-scheduling\AIMMSProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2971D9A6-5A8A-45FF-B390-096775F056B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA6F5A3-5A42-4A1F-B3F6-ACC91E71038A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25920" yWindow="2985" windowWidth="17280" windowHeight="9960" tabRatio="948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="55020" yWindow="-2490" windowWidth="21030" windowHeight="10395" tabRatio="948" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Horizon" sheetId="9" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="240">
   <si>
     <t>Port of Origin</t>
   </si>
@@ -135,9 +135,6 @@
   </si>
   <si>
     <t>Can Tho,Vietnam</t>
-  </si>
-  <si>
-    <t>Lamu Mainland</t>
   </si>
   <si>
     <t>2023-09-08</t>
@@ -1117,10 +1114,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1128,7 +1125,7 @@
         <v>45069</v>
       </c>
       <c r="B2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -1154,7 +1151,7 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1173,7 +1170,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C3">
         <v>184</v>
@@ -1181,10 +1178,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" t="s">
         <v>82</v>
-      </c>
-      <c r="B4" t="s">
-        <v>83</v>
       </c>
       <c r="C4">
         <v>70</v>
@@ -1192,10 +1189,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C5">
         <v>189</v>
@@ -1203,10 +1200,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6">
         <v>164</v>
@@ -1232,7 +1229,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
@@ -1241,7 +1238,7 @@
         <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E1" t="s">
         <v>5</v>
@@ -1250,7 +1247,7 @@
         <v>6</v>
       </c>
       <c r="G1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -1353,16 +1350,16 @@
         <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="D6">
         <v>1121000</v>
       </c>
       <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
         <v>34</v>
-      </c>
-      <c r="F6" t="s">
-        <v>35</v>
       </c>
       <c r="G6">
         <v>178</v>
@@ -1370,22 +1367,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
         <v>36</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>37</v>
-      </c>
-      <c r="C7" t="s">
-        <v>38</v>
       </c>
       <c r="D7">
         <v>1300600</v>
       </c>
       <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
         <v>39</v>
-      </c>
-      <c r="F7" t="s">
-        <v>40</v>
       </c>
       <c r="G7">
         <v>190</v>
@@ -1393,22 +1390,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" t="s">
         <v>41</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>42</v>
-      </c>
-      <c r="C8" t="s">
-        <v>43</v>
       </c>
       <c r="D8">
         <v>1275700</v>
       </c>
       <c r="E8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" t="s">
         <v>44</v>
-      </c>
-      <c r="F8" t="s">
-        <v>45</v>
       </c>
       <c r="G8">
         <v>52</v>
@@ -1416,22 +1413,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
         <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D9">
         <v>1057000</v>
       </c>
       <c r="E9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" t="s">
         <v>48</v>
-      </c>
-      <c r="F9" t="s">
-        <v>49</v>
       </c>
       <c r="G9">
         <v>87</v>
@@ -1439,22 +1436,22 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" t="s">
         <v>50</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>51</v>
-      </c>
-      <c r="C10" t="s">
-        <v>52</v>
       </c>
       <c r="D10">
         <v>1890000</v>
       </c>
       <c r="E10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" t="s">
         <v>53</v>
-      </c>
-      <c r="F10" t="s">
-        <v>54</v>
       </c>
       <c r="G10">
         <v>166</v>
@@ -1462,22 +1459,22 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
         <v>55</v>
       </c>
-      <c r="B11" t="s">
-        <v>56</v>
-      </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11">
         <v>1630900</v>
       </c>
       <c r="E11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" t="s">
         <v>57</v>
-      </c>
-      <c r="F11" t="s">
-        <v>58</v>
       </c>
       <c r="G11">
         <v>130</v>
@@ -1485,22 +1482,22 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" t="s">
         <v>59</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>60</v>
-      </c>
-      <c r="C12" t="s">
-        <v>61</v>
       </c>
       <c r="D12">
         <v>1181100</v>
       </c>
       <c r="E12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G12">
         <v>80</v>
@@ -1508,22 +1505,22 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" t="s">
         <v>63</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>64</v>
-      </c>
-      <c r="C13" t="s">
-        <v>65</v>
       </c>
       <c r="D13">
         <v>1465100</v>
       </c>
       <c r="E13" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" t="s">
         <v>66</v>
-      </c>
-      <c r="F13" t="s">
-        <v>67</v>
       </c>
       <c r="G13">
         <v>61</v>
@@ -1531,22 +1528,22 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" t="s">
         <v>68</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>69</v>
-      </c>
-      <c r="C14" t="s">
-        <v>70</v>
       </c>
       <c r="D14">
         <v>1204100</v>
       </c>
       <c r="E14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" t="s">
         <v>71</v>
-      </c>
-      <c r="F14" t="s">
-        <v>72</v>
       </c>
       <c r="G14">
         <v>178</v>
@@ -1554,22 +1551,22 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" t="s">
         <v>73</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>74</v>
-      </c>
-      <c r="C15" t="s">
-        <v>75</v>
       </c>
       <c r="D15">
         <v>1190600</v>
       </c>
       <c r="E15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G15">
         <v>190</v>
@@ -1577,22 +1574,22 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" t="s">
         <v>77</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>78</v>
-      </c>
-      <c r="C16" t="s">
-        <v>79</v>
       </c>
       <c r="D16">
         <v>1394300</v>
       </c>
       <c r="E16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G16">
         <v>52</v>
@@ -1605,7 +1602,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F178"/>
+  <dimension ref="A1:F176"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.6640625" bestFit="1" customWidth="1"/>
@@ -1627,15 +1624,15 @@
         <v>9</v>
       </c>
       <c r="E1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F1" t="s">
         <v>234</v>
-      </c>
-      <c r="F1" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B2">
         <v>22.488900000000001</v>
@@ -1655,7 +1652,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B3">
         <v>-8.0555555559999998</v>
@@ -1675,7 +1672,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B4">
         <v>-3.5336110000000001</v>
@@ -1695,7 +1692,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B5">
         <v>-2.5649999999999999</v>
@@ -1715,7 +1712,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B6">
         <v>-20.7884999999999</v>
@@ -1735,7 +1732,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B7">
         <v>11.069476</v>
@@ -1755,7 +1752,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B8">
         <v>4.7387639999999998</v>
@@ -1775,7 +1772,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B9">
         <v>5.2892400000000004</v>
@@ -1795,7 +1792,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B10">
         <v>18.419934999999899</v>
@@ -1815,7 +1812,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B11">
         <v>13.921932</v>
@@ -1835,7 +1832,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B12">
         <v>18.949947099999999</v>
@@ -1855,7 +1852,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B13">
         <v>15.413885000000001</v>
@@ -1875,7 +1872,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B14">
         <v>8.5631989999999991</v>
@@ -1895,7 +1892,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B15">
         <v>-3.292189</v>
@@ -1915,7 +1912,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B16">
         <v>24.774781000000001</v>
@@ -1935,7 +1932,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B17">
         <v>-6.7410550000000002</v>
@@ -1955,7 +1952,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B18">
         <v>-15.258332999999899</v>
@@ -1975,7 +1972,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B19">
         <v>6.0935870000000003</v>
@@ -1995,7 +1992,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B20">
         <v>-4.7888380000000002</v>
@@ -2015,7 +2012,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B21">
         <v>-33.806725</v>
@@ -2035,7 +2032,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B22">
         <v>46.649510999999897</v>
@@ -2055,7 +2052,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B23">
         <v>46.329355999999898</v>
@@ -2075,7 +2072,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B24">
         <v>10.5389839999999</v>
@@ -2095,7 +2092,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B25">
         <v>10.028922999999899</v>
@@ -2135,7 +2132,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B27">
         <v>17.970659999999999</v>
@@ -2155,7 +2152,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B28">
         <v>22.392150000000001</v>
@@ -2175,7 +2172,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B29">
         <v>19.1809499999999</v>
@@ -2195,7 +2192,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B30">
         <v>13.5927799999999</v>
@@ -2215,7 +2212,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B31">
         <v>15.7277799999999</v>
@@ -2235,7 +2232,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B32">
         <v>15.59981</v>
@@ -2255,7 +2252,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B33">
         <v>15.825620000000001</v>
@@ -2275,7 +2272,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B34">
         <v>12.4825</v>
@@ -2315,7 +2312,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B36">
         <v>9.99073999999999</v>
@@ -2335,7 +2332,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B37">
         <v>-4.5772199999999996</v>
@@ -2355,7 +2352,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B38">
         <v>-5.0891699999999904</v>
@@ -2375,7 +2372,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B39">
         <v>9.3522199999999902</v>
@@ -2395,7 +2392,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B40">
         <v>9.3545099999999994</v>
@@ -2415,7 +2412,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B41">
         <v>-2.1961599999999999</v>
@@ -2455,7 +2452,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B43">
         <v>26.5333299999999</v>
@@ -2475,7 +2472,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B44">
         <v>-12.05659</v>
@@ -2495,7 +2492,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B45">
         <v>3.8801000000000001</v>
@@ -2515,7 +2512,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B46">
         <v>17.937379999999902</v>
@@ -2535,7 +2532,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B47">
         <v>10.39972</v>
@@ -2555,7 +2552,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B48">
         <v>10.9685399999999</v>
@@ -2575,7 +2572,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B49">
         <v>11.240789999999899</v>
@@ -2595,7 +2592,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B50">
         <v>18.543489999999899</v>
@@ -2615,7 +2612,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B51">
         <v>-16.996389999999899</v>
@@ -2635,7 +2632,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B52">
         <v>12.241070000000001</v>
@@ -2655,7 +2652,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B53">
         <v>-33.036000000000001</v>
@@ -2675,7 +2672,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B54">
         <v>-33.594729999999899</v>
@@ -2695,7 +2692,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B55">
         <v>-27.088859999999901</v>
@@ -2715,7 +2712,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B56">
         <v>-27.06812</v>
@@ -2735,7 +2732,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B57">
         <v>-26.342979999999901</v>
@@ -2755,7 +2752,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B58">
         <v>-38.719589999999997</v>
@@ -2775,7 +2772,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B59">
         <v>-32.946820000000002</v>
@@ -2795,7 +2792,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B60">
         <v>-38.554499999999898</v>
@@ -2815,7 +2812,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B61">
         <v>-34.613149999999898</v>
@@ -2835,7 +2832,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B62">
         <v>-34.92145</v>
@@ -2855,7 +2852,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B63">
         <v>-34.903280000000002</v>
@@ -2875,7 +2872,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B64">
         <v>-25.427779999999899</v>
@@ -2895,7 +2892,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B65">
         <v>-28.466670000000001</v>
@@ -2915,7 +2912,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B66">
         <v>-26.907779999999899</v>
@@ -2935,7 +2932,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B67">
         <v>-26.11694</v>
@@ -2955,7 +2952,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B68">
         <v>-25.5162599999999</v>
@@ -2975,7 +2972,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B69">
         <v>-23.960829999999898</v>
@@ -2995,7 +2992,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B70">
         <v>-22.979310000000002</v>
@@ -3015,7 +3012,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B71">
         <v>-22.906420000000001</v>
@@ -3035,7 +3032,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B72">
         <v>-22.906420000000001</v>
@@ -3055,7 +3052,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B73">
         <v>-12.971109999999999</v>
@@ -3075,7 +3072,7 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B74">
         <v>14.6937</v>
@@ -3095,7 +3092,7 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B75">
         <v>20.941879999999902</v>
@@ -3135,7 +3132,7 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B77">
         <v>10.65</v>
@@ -3155,7 +3152,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B78">
         <v>9.5379500000000004</v>
@@ -3175,7 +3172,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B79">
         <v>8.4871400000000001</v>
@@ -3195,7 +3192,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B80">
         <v>6.3005399999999998</v>
@@ -3215,7 +3212,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B81">
         <v>5.8769299999999998</v>
@@ -3235,7 +3232,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B82">
         <v>30.420179999999899</v>
@@ -3255,7 +3252,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B83">
         <v>35.767270000000003</v>
@@ -3275,7 +3272,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B84">
         <v>4.8981599999999998</v>
@@ -3295,7 +3292,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B85">
         <v>5.6698000000000004</v>
@@ -3315,7 +3312,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B86">
         <v>6.1287399999999996</v>
@@ -3335,7 +3332,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B87">
         <v>36.510759999999912</v>
@@ -3355,7 +3352,7 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B88">
         <v>6.3653599999999999</v>
@@ -3395,7 +3392,7 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B90">
         <v>6.4540699999999998</v>
@@ -3415,7 +3412,7 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B91">
         <v>0.29122999999999999</v>
@@ -3435,7 +3432,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B92">
         <v>4.0482699999999996</v>
@@ -3455,7 +3452,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B93">
         <v>2.9372500000000001</v>
@@ -3475,7 +3472,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B94">
         <v>36.769459999999903</v>
@@ -3495,7 +3492,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B95">
         <v>-8.8368199999999906</v>
@@ -3535,7 +3532,7 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B97">
         <v>-22.9575</v>
@@ -3555,7 +3552,7 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B98">
         <v>43.056109999999897</v>
@@ -3575,7 +3572,7 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B99">
         <v>-33.011670000000002</v>
@@ -3595,7 +3592,7 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B100">
         <v>-33.925840000000001</v>
@@ -3615,7 +3612,7 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B101">
         <v>41.323549999999898</v>
@@ -3635,7 +3632,7 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B102">
         <v>32.11486</v>
@@ -3655,7 +3652,7 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B103">
         <v>40.98272</v>
@@ -3675,7 +3672,7 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B104">
         <v>31.201759999999901</v>
@@ -3695,7 +3692,7 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B105">
         <v>46.299140000000001</v>
@@ -3715,7 +3712,7 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B106">
         <v>46.485720000000001</v>
@@ -3735,7 +3732,7 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B107">
         <v>-29.857900000000001</v>
@@ -3755,7 +3752,7 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B108">
         <v>46.965910000000001</v>
@@ -3795,7 +3792,7 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B110">
         <v>31.2653099999999</v>
@@ -3815,7 +3812,7 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B111">
         <v>-25.962219999999999</v>
@@ -3835,7 +3832,7 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B112">
         <v>-25.965529999999902</v>
@@ -3855,7 +3852,7 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B113">
         <v>68.979169999999897</v>
@@ -3875,7 +3872,7 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B114">
         <v>36.811959999999907</v>
@@ -3895,7 +3892,7 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B115">
         <v>-19.843610000000002</v>
@@ -3915,7 +3912,7 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B116">
         <v>29.526669999999999</v>
@@ -3935,7 +3932,7 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B117">
         <v>33.893320000000003</v>
@@ -3955,7 +3952,7 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B118">
         <v>34.433520000000001</v>
@@ -3975,7 +3972,7 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B119">
         <v>34.507800000000003</v>
@@ -3995,7 +3992,7 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B120">
         <v>55.81353</v>
@@ -4015,7 +4012,7 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B121">
         <v>44.72439</v>
@@ -4035,7 +4032,7 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B122">
         <v>-6.8234899999999996</v>
@@ -4055,7 +4052,7 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B123">
         <v>-4.0546600000000002</v>
@@ -4075,7 +4072,7 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B124">
         <v>47.231349999999892</v>
@@ -4095,7 +4092,7 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B125">
         <v>41.64228</v>
@@ -4115,7 +4112,7 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B126">
         <v>42.142719999999997</v>
@@ -4135,7 +4132,7 @@
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B127">
         <v>-0.35816999999999999</v>
@@ -4155,7 +4152,7 @@
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B128">
         <v>11.58901</v>
@@ -4175,7 +4172,7 @@
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B129">
         <v>-11.702159999999999</v>
@@ -4195,7 +4192,7 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B130">
         <v>-12.16672</v>
@@ -4215,7 +4212,7 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B131">
         <v>10.4395899999999</v>
@@ -4235,7 +4232,7 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B132">
         <v>2.0371100000000002</v>
@@ -4255,7 +4252,7 @@
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B133">
         <v>-18.1492</v>
@@ -4275,7 +4272,7 @@
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B134">
         <v>-4.6200099999999997</v>
@@ -4295,7 +4292,7 @@
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B135">
         <v>-4.6200099999999997</v>
@@ -4315,7 +4312,7 @@
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B136">
         <v>-20.161939999999898</v>
@@ -4335,7 +4332,7 @@
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B137">
         <v>24.860800000000001</v>
@@ -4355,7 +4352,7 @@
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B138">
         <v>23.0333299999999</v>
@@ -4375,7 +4372,7 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B139">
         <v>19.07283</v>
@@ -4395,7 +4392,7 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B140">
         <v>4.1752099999999999</v>
@@ -4415,7 +4412,7 @@
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B141">
         <v>12.91723</v>
@@ -4435,7 +4432,7 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B142">
         <v>11.24802</v>
@@ -4455,7 +4452,7 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B143">
         <v>9.9398800000000005</v>
@@ -4475,7 +4472,7 @@
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B144">
         <v>8.8811300000000006</v>
@@ -4495,7 +4492,7 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B145">
         <v>8.7673500000000004</v>
@@ -4515,7 +4512,7 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B146">
         <v>6.9354800000000001</v>
@@ -4535,7 +4532,7 @@
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B147">
         <v>13.08784</v>
@@ -4555,7 +4552,7 @@
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B148">
         <v>13.24751</v>
@@ -4575,7 +4572,7 @@
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B149">
         <v>16.960360000000001</v>
@@ -4595,7 +4592,7 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B150">
         <v>17.68009</v>
@@ -4615,7 +4612,7 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B151">
         <v>20.316410000000001</v>
@@ -4635,7 +4632,7 @@
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B152">
         <v>22.562629999999899</v>
@@ -4655,7 +4652,7 @@
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B153">
         <v>22.3384</v>
@@ -4675,7 +4672,7 @@
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B154">
         <v>16.80528</v>
@@ -4695,7 +4692,7 @@
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B155">
         <v>16.661100000000001</v>
@@ -4715,7 +4712,7 @@
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B156">
         <v>3.7755000000000001</v>
@@ -4735,7 +4732,7 @@
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B157">
         <v>-2.0301</v>
@@ -4755,7 +4752,7 @@
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B158">
         <v>10.60932</v>
@@ -4795,7 +4792,7 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B160">
         <v>10.82302</v>
@@ -4815,7 +4812,7 @@
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B161">
         <v>20.864809999999999</v>
@@ -4835,7 +4832,7 @@
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B162">
         <v>16.0677799999999</v>
@@ -4855,7 +4852,7 @@
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B163">
         <v>13.7764799999999</v>
@@ -4875,7 +4872,7 @@
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B164">
         <v>-3.3198699999999999</v>
@@ -4895,7 +4892,7 @@
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B165">
         <v>-1.26753</v>
@@ -4915,7 +4912,7 @@
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B166">
         <v>-5.1486099999999997</v>
@@ -4935,7 +4932,7 @@
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B167">
         <v>14.604200000000001</v>
@@ -4955,7 +4952,7 @@
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B168">
         <v>6.9102800000000002</v>
@@ -4975,7 +4972,7 @@
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B169">
         <v>8.1480999999999906</v>
@@ -4995,7 +4992,7 @@
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B170">
         <v>10.31672</v>
@@ -5035,7 +5032,7 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B172">
         <v>8.4822199999999999</v>
@@ -5055,7 +5052,7 @@
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B173">
         <v>8.9472199999999997</v>
@@ -5075,7 +5072,7 @@
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B174">
         <v>9.7889999999999997</v>
@@ -5095,7 +5092,7 @@
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B175">
         <v>7.0730599999999999</v>
@@ -5115,7 +5112,7 @@
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B176">
         <v>-9.4772300000000005</v>
@@ -5131,22 +5128,6 @@
       </c>
       <c r="F176">
         <v>2687</v>
-      </c>
-    </row>
-    <row r="177" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E177">
-        <v>379</v>
-      </c>
-      <c r="F177">
-        <v>2499</v>
-      </c>
-    </row>
-    <row r="178" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E178">
-        <v>304</v>
-      </c>
-      <c r="F178">
-        <v>3763</v>
       </c>
     </row>
   </sheetData>

</xml_diff>